<commit_message>
Implemented ai and algorithm
</commit_message>
<xml_diff>
--- a/output/corroboria_report.xlsx
+++ b/output/corroboria_report.xlsx
@@ -12,12 +12,18 @@
     <sheet name="Écarts justifiés" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Rapport complet" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="File IA" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Analyse IA" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Priorisation IA" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Patterns IA" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'À investiguer'!$A$1:$L$77</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Écarts justifiés'!$A$1:$H$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rapport complet'!$A$1:$Y$503</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'File IA'!$A$1:$Y$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Analyse IA'!$A$1:$Q$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Priorisation IA'!$A$1:$N$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Patterns IA'!$A$1:$I$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,9 +31,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -42,7 +47,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +57,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007030A0"/>
       </patternFill>
     </fill>
   </fills>
@@ -67,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -76,8 +86,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -628,7 +644,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -5197,7 +5212,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="5" t="n">
         <v>34739</v>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -5237,7 +5252,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="5" t="n">
         <v>43079</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -5277,7 +5292,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="5" t="n">
         <v>33893</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -5317,7 +5332,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="5" t="n">
         <v>38025</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -5357,7 +5372,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="5" t="n">
         <v>31593</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -5397,7 +5412,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="5" t="n">
         <v>35220</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -5437,7 +5452,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="5" t="n">
         <v>34776</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -5477,7 +5492,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="5" t="n">
         <v>42087</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -5517,7 +5532,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="5" t="n">
         <v>34253</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -5557,7 +5572,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="5" t="n">
         <v>39227</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -5597,7 +5612,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="5" t="n">
         <v>39250</v>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -5637,7 +5652,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="5" t="n">
         <v>42083</v>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -5677,7 +5692,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" s="5" t="n">
         <v>31228</v>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -5717,7 +5732,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="5" t="n">
         <v>34778</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -5757,7 +5772,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D16" s="5" t="n">
         <v>40174</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -5797,7 +5812,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" s="5" t="n">
         <v>36614</v>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -5837,7 +5852,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="D18" s="5" t="n">
         <v>32880</v>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -5877,7 +5892,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="D19" s="5" t="n">
         <v>31291</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -5917,7 +5932,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D20" s="4" t="n">
+      <c r="D20" s="5" t="n">
         <v>32770</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -5957,7 +5972,7 @@
           <t>onboardDate</t>
         </is>
       </c>
-      <c r="D21" s="4" t="n">
+      <c r="D21" s="5" t="n">
         <v>37967</v>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -6255,7 +6270,7 @@
           <t>1964-08-15</t>
         </is>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="J3" s="5" t="n">
         <v>42461</v>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -6451,7 +6466,7 @@
           <t>1997-06-24</t>
         </is>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="J5" s="5" t="n">
         <v>43584</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -6647,7 +6662,7 @@
           <t>1970-02-10</t>
         </is>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="J7" s="5" t="n">
         <v>36927</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -6843,7 +6858,7 @@
           <t>1955-07-06</t>
         </is>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="J9" s="5" t="n">
         <v>39902</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -7039,7 +7054,7 @@
           <t>1984-09-22</t>
         </is>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="J11" s="5" t="n">
         <v>39902</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -7334,7 +7349,7 @@
           <t>1988-09-02</t>
         </is>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="J14" s="5" t="n">
         <v>36617</v>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -7708,7 +7723,7 @@
           <t>2001-11-16</t>
         </is>
       </c>
-      <c r="J18" s="4" t="n">
+      <c r="J18" s="5" t="n">
         <v>44839</v>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -8003,7 +8018,7 @@
           <t>1993-05-23</t>
         </is>
       </c>
-      <c r="J21" s="4" t="n">
+      <c r="J21" s="5" t="n">
         <v>42499</v>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -8464,7 +8479,7 @@
           <t>2001-02-05</t>
         </is>
       </c>
-      <c r="J26" s="4" t="n">
+      <c r="J26" s="5" t="n">
         <v>41567</v>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -8840,7 +8855,7 @@
           <t>1950-08-09</t>
         </is>
       </c>
-      <c r="J30" s="4" t="n">
+      <c r="J30" s="5" t="n">
         <v>45740</v>
       </c>
       <c r="K30" s="3" t="inlineStr">
@@ -9135,7 +9150,7 @@
           <t>1969-04-04</t>
         </is>
       </c>
-      <c r="J33" s="4" t="n">
+      <c r="J33" s="5" t="n">
         <v>39902</v>
       </c>
       <c r="K33" s="3" t="inlineStr">
@@ -9331,7 +9346,7 @@
           <t>1960-12-04</t>
         </is>
       </c>
-      <c r="J35" s="4" t="n">
+      <c r="J35" s="5" t="n">
         <v>44970</v>
       </c>
       <c r="K35" s="3" t="inlineStr">
@@ -9626,7 +9641,7 @@
           <t>1987-01-12</t>
         </is>
       </c>
-      <c r="J38" s="4" t="n">
+      <c r="J38" s="5" t="n">
         <v>39902</v>
       </c>
       <c r="K38" s="3" t="inlineStr">
@@ -9822,7 +9837,7 @@
           <t>1980-10-09</t>
         </is>
       </c>
-      <c r="J40" s="4" t="n">
+      <c r="J40" s="5" t="n">
         <v>40000</v>
       </c>
       <c r="K40" s="3" t="inlineStr">
@@ -10018,7 +10033,7 @@
           <t>1981-06-17</t>
         </is>
       </c>
-      <c r="J42" s="4" t="n">
+      <c r="J42" s="5" t="n">
         <v>45950</v>
       </c>
       <c r="K42" s="3" t="inlineStr">
@@ -10313,7 +10328,7 @@
           <t>1971-05-19</t>
         </is>
       </c>
-      <c r="J45" s="4" t="n">
+      <c r="J45" s="5" t="n">
         <v>39902</v>
       </c>
       <c r="K45" s="3" t="inlineStr">
@@ -10509,7 +10524,7 @@
           <t>1971-02-13</t>
         </is>
       </c>
-      <c r="J47" s="4" t="n">
+      <c r="J47" s="5" t="n">
         <v>42086</v>
       </c>
       <c r="K47" s="3" t="inlineStr">
@@ -10885,7 +10900,7 @@
           <t>1968-02-04</t>
         </is>
       </c>
-      <c r="J51" s="4" t="n">
+      <c r="J51" s="5" t="n">
         <v>39902</v>
       </c>
       <c r="K51" s="3" t="inlineStr">
@@ -11081,7 +11096,7 @@
           <t>1987-08-19</t>
         </is>
       </c>
-      <c r="J53" s="4" t="n">
+      <c r="J53" s="5" t="n">
         <v>36927</v>
       </c>
       <c r="K53" s="3" t="inlineStr">
@@ -11277,7 +11292,7 @@
           <t>2003-06-18</t>
         </is>
       </c>
-      <c r="J55" s="4" t="n">
+      <c r="J55" s="5" t="n">
         <v>44285</v>
       </c>
       <c r="K55" s="3" t="inlineStr">
@@ -13603,7 +13618,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G78" s="4" t="n">
+      <c r="G78" s="5" t="n">
         <v>34739</v>
       </c>
       <c r="H78" s="3" t="inlineStr">
@@ -13700,7 +13715,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G79" s="4" t="n">
+      <c r="G79" s="5" t="n">
         <v>43079</v>
       </c>
       <c r="H79" s="3" t="inlineStr">
@@ -13797,7 +13812,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G80" s="4" t="n">
+      <c r="G80" s="5" t="n">
         <v>33893</v>
       </c>
       <c r="H80" s="3" t="inlineStr">
@@ -13894,7 +13909,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G81" s="4" t="n">
+      <c r="G81" s="5" t="n">
         <v>38025</v>
       </c>
       <c r="H81" s="3" t="inlineStr">
@@ -13991,7 +14006,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G82" s="4" t="n">
+      <c r="G82" s="5" t="n">
         <v>31593</v>
       </c>
       <c r="H82" s="3" t="inlineStr">
@@ -14088,7 +14103,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G83" s="4" t="n">
+      <c r="G83" s="5" t="n">
         <v>35220</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
@@ -14185,7 +14200,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G84" s="4" t="n">
+      <c r="G84" s="5" t="n">
         <v>34776</v>
       </c>
       <c r="H84" s="3" t="inlineStr">
@@ -14282,7 +14297,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G85" s="4" t="n">
+      <c r="G85" s="5" t="n">
         <v>42087</v>
       </c>
       <c r="H85" s="3" t="inlineStr">
@@ -14379,7 +14394,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G86" s="4" t="n">
+      <c r="G86" s="5" t="n">
         <v>34253</v>
       </c>
       <c r="H86" s="3" t="inlineStr">
@@ -14476,7 +14491,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G87" s="4" t="n">
+      <c r="G87" s="5" t="n">
         <v>39227</v>
       </c>
       <c r="H87" s="3" t="inlineStr">
@@ -14573,7 +14588,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G88" s="4" t="n">
+      <c r="G88" s="5" t="n">
         <v>39250</v>
       </c>
       <c r="H88" s="3" t="inlineStr">
@@ -14670,7 +14685,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G89" s="4" t="n">
+      <c r="G89" s="5" t="n">
         <v>42083</v>
       </c>
       <c r="H89" s="3" t="inlineStr">
@@ -14767,7 +14782,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G90" s="4" t="n">
+      <c r="G90" s="5" t="n">
         <v>31228</v>
       </c>
       <c r="H90" s="3" t="inlineStr">
@@ -14864,7 +14879,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G91" s="4" t="n">
+      <c r="G91" s="5" t="n">
         <v>34778</v>
       </c>
       <c r="H91" s="3" t="inlineStr">
@@ -14961,7 +14976,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G92" s="4" t="n">
+      <c r="G92" s="5" t="n">
         <v>40174</v>
       </c>
       <c r="H92" s="3" t="inlineStr">
@@ -15058,7 +15073,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G93" s="4" t="n">
+      <c r="G93" s="5" t="n">
         <v>36614</v>
       </c>
       <c r="H93" s="3" t="inlineStr">
@@ -15155,7 +15170,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G94" s="4" t="n">
+      <c r="G94" s="5" t="n">
         <v>32880</v>
       </c>
       <c r="H94" s="3" t="inlineStr">
@@ -15252,7 +15267,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G95" s="4" t="n">
+      <c r="G95" s="5" t="n">
         <v>31291</v>
       </c>
       <c r="H95" s="3" t="inlineStr">
@@ -15349,7 +15364,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G96" s="4" t="n">
+      <c r="G96" s="5" t="n">
         <v>32770</v>
       </c>
       <c r="H96" s="3" t="inlineStr">
@@ -15446,7 +15461,7 @@
           <t>DateEmbaucheRécente</t>
         </is>
       </c>
-      <c r="G97" s="4" t="n">
+      <c r="G97" s="5" t="n">
         <v>37967</v>
       </c>
       <c r="H97" s="3" t="inlineStr">
@@ -25896,7 +25911,7 @@
           <t>2010-05-28</t>
         </is>
       </c>
-      <c r="J208" s="4" t="n">
+      <c r="J208" s="5" t="n">
         <v>40326</v>
       </c>
       <c r="K208" s="3" t="inlineStr">
@@ -44726,7 +44741,7 @@
           <t>2015-06-17</t>
         </is>
       </c>
-      <c r="J408" s="4" t="n">
+      <c r="J408" s="5" t="n">
         <v>42172</v>
       </c>
       <c r="K408" s="3" t="inlineStr">
@@ -53996,4 +54011,1918 @@
   <autoFilter ref="A1:Y2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="25" customWidth="1" min="14" max="14"/>
+    <col width="25" customWidth="1" min="15" max="15"/>
+    <col width="45" customWidth="1" min="16" max="16"/>
+    <col width="23" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>employee_id</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>assignment_type</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>source_row_index</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>destination_row_index</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>pair_match_score</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>selected_by_best_matching</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>best_matching_score</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>second_matching_score</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>matching_confidence</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>matching_margin</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>recommendation</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>recommended_action</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>evidence_summary</t>
+        </is>
+      </c>
+      <c r="N1" s="6" t="inlineStr">
+        <is>
+          <t>training_positive_count</t>
+        </is>
+      </c>
+      <c r="O1" s="6" t="inlineStr">
+        <is>
+          <t>training_negative_count</t>
+        </is>
+      </c>
+      <c r="P1" s="6" t="inlineStr">
+        <is>
+          <t>ai_method</t>
+        </is>
+      </c>
+      <c r="Q1" s="6" t="inlineStr">
+        <is>
+          <t>deterministic_verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>7683990</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.7808310000000001</v>
+      </c>
+      <c r="F2" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.7808310000000001</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0.031143</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0.962</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0.749688</v>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>PROPOSITION_IA</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Cette paire appartient à la meilleure combinaison biunivoque trouvée par le modèle. Valider fonctionnellement avant acceptation.</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Correspondances: positionId, positionCode, siteCode, divisionId, divisionCode, payGradeId, type d'affectation. écart heures/semaine=0. écart heures/jour=0.</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier + optimisation de correspondance biunivoque</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>A_INVESTIGUER</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>7683990</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.7808310000000001</v>
+      </c>
+      <c r="F3" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0.7808310000000001</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.031143</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0.962</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0.749688</v>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>PROPOSITION_IA</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Cette paire appartient à la meilleure combinaison biunivoque trouvée par le modèle. Valider fonctionnellement avant acceptation.</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Correspondances: positionId, positionCode, siteCode, divisionId, divisionCode, payGradeId, type d'affectation. écart heures/semaine=0. écart heures/jour=0.</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier + optimisation de correspondance biunivoque</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>A_INVESTIGUER</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>7683990</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.031143</v>
+      </c>
+      <c r="F4" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.7808310000000001</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0.031143</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>0.962</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0.749688</v>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>CANDIDAT_ALTERNATIF</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Cette paire n'appartient pas à la meilleure combinaison globale.</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Correspondances: siteCode, divisionId, divisionCode, payGradeId, type d'affectation. Différences: positionId, positionCode. écart heures/semaine=0. écart heures/jour=0.</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier + optimisation de correspondance biunivoque</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>A_INVESTIGUER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>7683990</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.031143</v>
+      </c>
+      <c r="F5" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0.7808310000000001</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0.031143</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0.962</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0.749688</v>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>CANDIDAT_ALTERNATIF</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Cette paire n'appartient pas à la meilleure combinaison globale.</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Correspondances: siteCode, divisionId, divisionCode, payGradeId, type d'affectation. Différences: positionId, positionCode. écart heures/semaine=0. écart heures/jour=0.</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier + optimisation de correspondance biunivoque</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>A_INVESTIGUER</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Q5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>employee_id</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>anomaly_count</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>investigate_count</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>direct_anomaly_count</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>rule_anomaly_count</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>structural_anomaly_count</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>critical_count</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>high_priority_count</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>unique_anomaly_fields</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>mean_field_rarity</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>max_field_rarity</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>ai_anomaly_score</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>ai_priority</t>
+        </is>
+      </c>
+      <c r="N1" s="6" t="inlineStr">
+        <is>
+          <t>ai_explanation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>3712987</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0.4800000000000001</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>ÉLEVÉE</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=1.000. 2 écart(s) direct(s); plusieurs anomalies simultanées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>1545850</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0.3166666666666667</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>0.9968197659469824</v>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>CRITIQUE</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.997. anomalie structurelle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>7683990</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>0.7228588978658625</v>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.723. 2 écart(s) direct(s); plusieurs anomalies simultanées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2762457</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>0.345051321342558</v>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.345. profil proche des anomalies récurrentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>4625374</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>0.345051321342558</v>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.345. profil proche des anomalies récurrentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>7254364</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L7" s="3" t="n">
+        <v>0.345051321342558</v>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.345. profil proche des anomalies récurrentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>3241002</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>0.2935404914079955</v>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.294. 1 écart(s) direct(s).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>6035643</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L9" s="3" t="n">
+        <v>0.2935404914079955</v>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.294. 1 écart(s) direct(s).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2911996</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>0.2562094057764407</v>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.256. 2 écart(s) direct(s); plusieurs anomalies simultanées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>4402456</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L11" s="3" t="n">
+        <v>0.2562094057764407</v>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.256. 2 écart(s) direct(s); plusieurs anomalies simultanées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2173396</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.000. profil proche des anomalies récurrentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2648214</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.000. profil proche des anomalies récurrentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2747515</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.000. profil proche des anomalies récurrentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>4880692</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.000. profil proche des anomalies récurrentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>6783031</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.000. profil proche des anomalies récurrentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>7070325</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.000. profil proche des anomalies récurrentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>7603160</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.000. profil proche des anomalies récurrentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>8142123</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.000. profil proche des anomalies récurrentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>8644330</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.000. profil proche des anomalies récurrentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>9989151</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>FAIBLE</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>Score IA=0.000. profil proche des anomalies récurrentes.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N21"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>rule_id</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>decision_source</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>occurrences</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>affected_employees</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>employee_prevalence</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>pattern_type</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>ai_interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>assignmentStartDate</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>RULE_ASSIGNMENT_START</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>ANOMALIE</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>RULE</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEMATIQUE</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Écart observé sur une grande partie de la population. Vérifier en priorité une règle de transformation, une configuration globale ou une limite du jeu de données.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>contactEmail</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>RULE_EMAIL</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>A_INVESTIGUER</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>RULE_LIMITATION</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEMATIQUE</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Écart observé sur une grande partie de la population. Vérifier en priorité une règle de transformation, une configuration globale ou une limite du jeu de données.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>positionName</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>RULE_POSITION_NAME</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>ANOMALIE</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>RULE</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>SYSTEMATIQUE</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Écart observé sur une grande partie de la population. Vérifier en priorité une règle de transformation, une configuration globale ou une limite du jeu de données.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>contractTypeCode</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>RULE_CONTRACT_TYPE</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>ANOMALIE</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>RULE</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>RECURRENT</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Écart récurrent mais non généralisé. Rechercher une cause commune touchant un sous-ensemble d'employés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>dailyHoursOverride</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>ANOMALIE</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>RECURRENT</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Écart récurrent mais non généralisé. Rechercher une cause commune touchant un sous-ensemble d'employés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>weeklyHoursOverride</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>ANOMALIE</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>RECURRENT</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Écart récurrent mais non généralisé. Rechercher une cause commune touchant un sous-ensemble d'employés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>siteName</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>ANOMALIE</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>ISOLE</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Écart relativement isolé. Une investigation individuelle est probablement plus pertinente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>__ASSIGNMENT__</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>ANOMALIE</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>STRUCTURAL</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>ISOLE</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Écart relativement isolé. Une investigation individuelle est probablement plus pertinente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>__ASSIGNMENT__</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>A_INVESTIGUER</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>STRUCTURAL</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>ISOLE</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Écart relativement isolé. Une investigation individuelle est probablement plus pertinente.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>